<commit_message>
Atualiza informações de copyright e versão nos scripts e no README, e substitui o arquivo de dados de lançamento
</commit_message>
<xml_diff>
--- a/projeto/dados_lancamento.xlsx
+++ b/projeto/dados_lancamento.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\PortableApps\automacao-lancamento-financeiro\projeto\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\warre\Downloads\Portable Apps\automacao-lancamento-financeiro\projeto\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4D5496B5-FF51-4A1A-8FDB-B2671F711EFA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2AA35D2D-0CDB-4270-8191-7BE6FB026376}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{117D8EBC-9BC0-4629-86B5-E598CADE3FE5}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{117D8EBC-9BC0-4629-86B5-E598CADE3FE5}"/>
   </bookViews>
   <sheets>
     <sheet name="Planilha1" sheetId="1" r:id="rId1"/>
@@ -56,13 +56,13 @@
     <t>0880000912</t>
   </si>
   <si>
-    <t>10/2025</t>
-  </si>
-  <si>
-    <t>15/11/2025</t>
-  </si>
-  <si>
     <t>Teste automacao lancamento financeiro</t>
+  </si>
+  <si>
+    <t>03/2026</t>
+  </si>
+  <si>
+    <t>15/04/2026</t>
   </si>
 </sst>
 </file>
@@ -436,14 +436,14 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{991622FA-3BAB-49DA-88B6-F27855ED8650}">
   <dimension ref="A1:F3"/>
-  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="9.140625" style="1"/>
-    <col min="2" max="2" width="11.85546875" style="1" customWidth="1"/>
-    <col min="3" max="16384" width="9.140625" style="1"/>
+    <col min="1" max="1" width="9.109375" style="1"/>
+    <col min="2" max="2" width="11.88671875" style="1" customWidth="1"/>
+    <col min="3" max="16384" width="9.109375" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -451,19 +451,19 @@
         <v>4</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>1</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
         <v>0</v>
       </c>
@@ -471,19 +471,19 @@
         <v>4</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D2" s="1" t="s">
         <v>2</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
         <v>0</v>
       </c>
@@ -491,16 +491,16 @@
         <v>4</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D3" s="1" t="s">
         <v>3</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
   </sheetData>

</xml_diff>